<commit_message>
fix: add burst flow modes and responsive date picker
</commit_message>
<xml_diff>
--- a/data/uploads/zhuanhua_demo.xlsx
+++ b/data/uploads/zhuanhua_demo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28000" windowHeight="11740"/>
+    <workbookView windowWidth="26860" windowHeight="11740"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1297" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="761">
   <si>
     <t>日期</t>
   </si>
@@ -2207,7 +2207,7 @@
     <t>0.01185835</t>
   </si>
   <si>
-    <t>其他</t>
+    <t>爆量未加微</t>
   </si>
   <si>
     <t>8.70</t>
@@ -2244,6 +2244,75 @@
   </si>
   <si>
     <t>0.03803291</t>
+  </si>
+  <si>
+    <t>2026-08-14</t>
+  </si>
+  <si>
+    <t>483</t>
+  </si>
+  <si>
+    <t>3.63</t>
+  </si>
+  <si>
+    <t>0.00352331</t>
+  </si>
+  <si>
+    <t>0.01372783</t>
+  </si>
+  <si>
+    <t>1602</t>
+  </si>
+  <si>
+    <t>爆量再植课</t>
+  </si>
+  <si>
+    <t>959</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>8.88</t>
+  </si>
+  <si>
+    <t>0.00870876</t>
+  </si>
+  <si>
+    <t>0.03242933</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>1.66</t>
+  </si>
+  <si>
+    <t>0.00055502</t>
+  </si>
+  <si>
+    <t>0.00599700</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>5.78</t>
+  </si>
+  <si>
+    <t>0.00148116</t>
+  </si>
+  <si>
+    <t>0.02437310</t>
+  </si>
+  <si>
+    <t>8.50</t>
+  </si>
+  <si>
+    <t>0.01203753</t>
+  </si>
+  <si>
+    <t>0.02296521</t>
   </si>
 </sst>
 </file>
@@ -3258,7 +3327,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:V203"/>
+  <dimension ref="A1:V209"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="7" width="16.8173076923077" customWidth="1"/>
@@ -7684,6 +7753,138 @@
       </c>
       <c r="G203" s="1" t="s">
         <v>737</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7">
+      <c r="A204" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="D204" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="E204" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="F204" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="G204" s="1" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7">
+      <c r="A205" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B205" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C205" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="D205" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E205" s="1"/>
+      <c r="F205" s="1"/>
+      <c r="G205" s="1"/>
+    </row>
+    <row r="206" spans="1:7">
+      <c r="A206" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B206" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="C206" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="D206" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="E206" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="F206" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="G206" s="1" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7">
+      <c r="A207" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B207" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C207" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="D207" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="E207" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="F207" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="G207" s="1" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7">
+      <c r="A208" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B208" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C208" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D208" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="E208" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="F208" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="G208" s="1" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7">
+      <c r="A209" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="B209" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C209" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="D209" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E209" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="F209" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="G209" s="1" t="s">
+        <v>760</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add efficiency target data
</commit_message>
<xml_diff>
--- a/data/uploads/zhuanhua_demo.xlsx
+++ b/data/uploads/zhuanhua_demo.xlsx
@@ -10,7 +10,7 @@
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet!$A$1:$V$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet!$A$1:$V$228</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="454">
   <si>
     <t>日期</t>
   </si>
@@ -1320,19 +1320,92 @@
   </si>
   <si>
     <t>0.03450863</t>
+  </si>
+  <si>
+    <t>2026-08-18</t>
+  </si>
+  <si>
+    <t>504</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>3.50</t>
+  </si>
+  <si>
+    <t>0.00358578</t>
+  </si>
+  <si>
+    <t>0.01424977</t>
+  </si>
+  <si>
+    <t>1857</t>
+  </si>
+  <si>
+    <t>1260</t>
+  </si>
+  <si>
+    <t>138</t>
+  </si>
+  <si>
+    <t>9.13</t>
+  </si>
+  <si>
+    <t>0.01184044</t>
+  </si>
+  <si>
+    <t>0.03296358</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>2.50</t>
+  </si>
+  <si>
+    <t>0.00091684</t>
+  </si>
+  <si>
+    <t>0.01130506</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>15.29</t>
+  </si>
+  <si>
+    <t>0.02247427</t>
+  </si>
+  <si>
+    <t>0.04220907</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>20260820</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="[$-409]yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1357,9 +1430,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -1824,16 +1902,13 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1842,126 +1917,131 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2350,7 +2430,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:V218"/>
+  <dimension ref="A1:V233"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="7" width="16.8173076923077" customWidth="1"/>
@@ -6997,116 +7077,455 @@
       </c>
     </row>
     <row r="214" hidden="1" spans="1:7">
-      <c r="A214" s="6" t="s">
+      <c r="A214" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="B214" s="6" t="s">
+      <c r="B214" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C214" s="6" t="s">
+      <c r="C214" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="D214" s="6" t="s">
+      <c r="D214" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E214" s="6"/>
-      <c r="F214" s="6"/>
-      <c r="G214" s="6"/>
+      <c r="E214" s="3"/>
+      <c r="F214" s="3"/>
+      <c r="G214" s="3"/>
     </row>
     <row r="215" hidden="1" spans="1:7">
-      <c r="A215" s="6" t="s">
+      <c r="A215" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="B215" s="6" t="s">
+      <c r="B215" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="C215" s="6" t="s">
+      <c r="C215" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="D215" s="6" t="s">
+      <c r="D215" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="E215" s="6" t="s">
+      <c r="E215" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="F215" s="6" t="s">
+      <c r="F215" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="G215" s="6" t="s">
+      <c r="G215" s="3" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="216" hidden="1" spans="1:7">
-      <c r="A216" s="6" t="s">
+      <c r="A216" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="B216" s="6" t="s">
+      <c r="B216" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C216" s="6" t="s">
+      <c r="C216" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="D216" s="6" t="s">
+      <c r="D216" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="E216" s="6" t="s">
+      <c r="E216" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="F216" s="6" t="s">
+      <c r="F216" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="G216" s="6" t="s">
+      <c r="G216" s="3" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="217" spans="1:7">
-      <c r="A217" s="6" t="s">
+      <c r="A217" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="B217" s="6" t="s">
+      <c r="B217" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C217" s="6" t="s">
+      <c r="C217" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="D217" s="6" t="s">
+      <c r="D217" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E217" s="6"/>
-      <c r="F217" s="6"/>
-      <c r="G217" s="6"/>
+      <c r="E217" s="3"/>
+      <c r="F217" s="3"/>
+      <c r="G217" s="3"/>
     </row>
     <row r="218" spans="1:7">
-      <c r="A218" s="6" t="s">
+      <c r="A218" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="B218" s="6" t="s">
+      <c r="B218" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="C218" s="6" t="s">
+      <c r="C218" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="D218" s="6" t="s">
+      <c r="D218" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="E218" s="6" t="s">
+      <c r="E218" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="F218" s="6" t="s">
+      <c r="F218" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="G218" s="6" t="s">
+      <c r="G218" s="3" t="s">
         <v>429</v>
       </c>
     </row>
+    <row r="219" spans="1:7">
+      <c r="A219" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B219" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="D219" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="E219" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="F219" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="G219" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7">
+      <c r="A220" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B220" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="D220" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E220" s="3"/>
+      <c r="F220" s="3"/>
+      <c r="G220" s="3"/>
+    </row>
+    <row r="221" spans="1:7">
+      <c r="A221" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B221" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="D221" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="E221" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="G221" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7">
+      <c r="A222" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B222" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="D222" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="E222" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="G222" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7">
+      <c r="A223" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B223" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="D223" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="E223" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="G223" s="3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7">
+      <c r="A224" s="6">
+        <v>46253</v>
+      </c>
+      <c r="B224" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C224" s="7">
+        <v>481</v>
+      </c>
+      <c r="D224" s="7">
+        <v>141</v>
+      </c>
+      <c r="E224" s="7">
+        <v>3.4113475177305</v>
+      </c>
+      <c r="F224" s="7">
+        <v>0.00331749305119699</v>
+      </c>
+      <c r="G224" s="7">
+        <v>0.0149309327952817</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7">
+      <c r="A225" s="6">
+        <v>46253</v>
+      </c>
+      <c r="B225" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C225" s="7">
+        <v>817</v>
+      </c>
+      <c r="D225" s="7">
+        <v>0</v>
+      </c>
+      <c r="E225" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="F225" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="G225" s="7" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7">
+      <c r="A226" s="6">
+        <v>46253</v>
+      </c>
+      <c r="B226" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="C226" s="7">
+        <v>874</v>
+      </c>
+      <c r="D226" s="7">
+        <v>131</v>
+      </c>
+      <c r="E226" s="7">
+        <v>6.67175572519084</v>
+      </c>
+      <c r="F226" s="7">
+        <v>0.0060008513793719</v>
+      </c>
+      <c r="G226" s="7">
+        <v>0.0234876783746742</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7">
+      <c r="A227" s="6">
+        <v>46253</v>
+      </c>
+      <c r="B227" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C227" s="7">
+        <v>98</v>
+      </c>
+      <c r="D227" s="7">
+        <v>49</v>
+      </c>
+      <c r="E227" s="7">
+        <v>2</v>
+      </c>
+      <c r="F227" s="7">
+        <v>0.000834106442195572</v>
+      </c>
+      <c r="G227" s="7">
+        <v>0.00951548694047966</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7">
+      <c r="A228" s="6">
+        <v>46253</v>
+      </c>
+      <c r="B228" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="C228" s="7">
+        <v>97</v>
+      </c>
+      <c r="D228" s="7">
+        <v>8</v>
+      </c>
+      <c r="E228" s="7">
+        <v>12.125</v>
+      </c>
+      <c r="F228" s="7">
+        <v>0.0193844924060751</v>
+      </c>
+      <c r="G228" s="7">
+        <v>0.0355571847507331</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7">
+      <c r="A229" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B229" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C229" s="8">
+        <v>592</v>
+      </c>
+      <c r="D229" s="8">
+        <v>144</v>
+      </c>
+      <c r="E229" s="8">
+        <v>4.11111111111111</v>
+      </c>
+      <c r="F229" s="8">
+        <v>0.00336377014994915</v>
+      </c>
+      <c r="G229" s="8">
+        <v>0.0185970533722866</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7">
+      <c r="A230" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B230" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C230" s="8">
+        <v>1058</v>
+      </c>
+      <c r="D230" s="8">
+        <v>0</v>
+      </c>
+      <c r="E230" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="F230" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="G230" s="8" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7">
+      <c r="A231" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B231" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C231" s="8">
+        <v>126</v>
+      </c>
+      <c r="D231" s="8">
+        <v>50</v>
+      </c>
+      <c r="E231" s="8">
+        <v>2.52</v>
+      </c>
+      <c r="F231" s="8">
+        <v>0.000965916931143922</v>
+      </c>
+      <c r="G231" s="8">
+        <v>0.0119239140721113</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7">
+      <c r="A232" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B232" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="C232" s="8">
+        <v>84</v>
+      </c>
+      <c r="D232" s="8">
+        <v>8</v>
+      </c>
+      <c r="E232" s="8">
+        <v>10.5</v>
+      </c>
+      <c r="F232" s="8">
+        <v>0.0158371040723982</v>
+      </c>
+      <c r="G232" s="8">
+        <v>0.0313082370480805</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7">
+      <c r="A233" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="B233" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C233" s="8">
+        <v>903</v>
+      </c>
+      <c r="D233" s="8">
+        <v>136</v>
+      </c>
+      <c r="E233" s="8">
+        <v>6.63970588235294</v>
+      </c>
+      <c r="F233" s="8">
+        <v>0.00657506717053671</v>
+      </c>
+      <c r="G233" s="8">
+        <v>0.0230263157894737</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:V216" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:V228" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="1">
-      <filters>
-        <filter val="大神"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="大神"/>
+      </customFilters>
     </filterColumn>
-    <sortState ref="A2:V216">
+    <sortState ref="A1:V228">
       <sortCondition ref="A1" descending="1"/>
     </sortState>
     <extLst/>

</xml_diff>